<commit_message>
Cenarios 1/2/6: nota de rebalanceamento + HP de minion por tier + taticas + regras novas; planilha de inimigos atualizada; registro da sessao
</commit_message>
<xml_diff>
--- a/playtest/Marca-de-Sangue-Controle-de-Inimigos.xlsx
+++ b/playtest/Marca-de-Sangue-Controle-de-Inimigos.xlsx
@@ -518,7 +518,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A21"/>
+  <dimension ref="A1:A22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="115" customWidth="1" min="1" max="1"/>
@@ -616,36 +616,43 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Vida (PV): cada membro tem 10 PV. Ordem do dano: superficial → profundo → permanente. Um membro fica</t>
+          <t>Vida (PV) — MODELO NOVO (playtest 1): cada membro tem 10 espaços. Enche de dano → vira PROFUNDO</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>INCAPACITADO com 10 de dano profundo. Anote o total de dano no membro atingido.</t>
+          <t>(incapacitado; só cura com tratamento). Dano além disso → PERMANENTE. Todo dano recebido gera 1 fadiga/ponto.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>EXCEÇÃO — Colosso (Cenário 5): cada região aguenta 20 (o dobro). Use Cab=Cabeça-cristal, Tro=NÚCLEO,</t>
+          <t>HP de MINION (para o mestre): fraco = cai com 10 de dano total · médio = 20 · forte = 30.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
+          <t>EXCEÇÃO — Colosso (Cenário 5): cada região aguenta 20 (o dobro). Use Cab=Cabeça-cristal, Tro=NÚCLEO,</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
           <t>BD/BE=braços, PD/PE=Base. Vencer = 20 de dano no Núcleo (que só abre ao destruir um braço).</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="2" t="inlineStr"/>
-    </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
+      <c r="A21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
         <is>
           <t>Dica: dá para imprimir (paisagem) ou usar na tela. O cabeçalho e a coluna do nome ficam congelados ao rolar.</t>
         </is>

</xml_diff>